<commit_message>
Fix matchedQty to sum all PlanningResult rows, not just latest planDate
matchedQty should be the plain sum of quantity (PlanningResult column F)
over every row whose partNumber (column B) matches - no planDate
filtering. The earlier "latest planDate only" heuristic was wrong.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DphkeLXanAW8ZqwZHK1tS
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -522,10 +522,10 @@
         <v>0</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>404193</v>
+        <v>1269136</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>404193</v>
+        <v>1269136</v>
       </c>
     </row>
     <row r="7">
@@ -554,10 +554,10 @@
         <v>636322.097301</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>395564</v>
+        <v>857390</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>-240758.097301</v>
+        <v>221067.902699</v>
       </c>
     </row>
     <row r="9">
@@ -618,10 +618,10 @@
         <v>640362.403425</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>402758</v>
+        <v>503515</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>-237604.403425</v>
+        <v>-136847.403425</v>
       </c>
     </row>
     <row r="13">
@@ -682,10 +682,10 @@
         <v>549918.708952</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>101295</v>
+        <v>456515</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>-448623.708952</v>
+        <v>-93403.70895200002</v>
       </c>
     </row>
     <row r="17">
@@ -714,10 +714,10 @@
         <v>44748.0079</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>40584</v>
+        <v>100225</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>-4164.007899999997</v>
+        <v>55476.9921</v>
       </c>
     </row>
     <row r="19">
@@ -922,10 +922,10 @@
         <v>48497.818672</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>432719</v>
+        <v>1065023</v>
       </c>
       <c r="D31" s="1" t="n">
-        <v>384221.181328</v>
+        <v>1016525.181328</v>
       </c>
     </row>
     <row r="32">
@@ -954,10 +954,10 @@
         <v>0</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>167837</v>
+        <v>268459</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>167837</v>
+        <v>268459</v>
       </c>
     </row>
     <row r="34">
@@ -970,10 +970,10 @@
         <v>0</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>166479</v>
+        <v>499420</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>166479</v>
+        <v>499420</v>
       </c>
     </row>
     <row r="35">
@@ -1003,7 +1003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1101,288 +1101,256 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T520D337M006ATE009</t>
+          <t>T520D477M004ATE010</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>636322.097301</v>
+        <v>181559.085912</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>395564</v>
+        <v>164687</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>-240758.097301</v>
+        <v>-16872.08591199998</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T520D477M004ATE010</t>
+          <t>T520D337M006ATE040</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>181559.085912</v>
+        <v>9048.833817999999</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>164687</v>
+        <v>0</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>-16872.08591199998</v>
+        <v>-9048.833817999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T520D337M006ATE040</t>
+          <t>T521V107M016ATE050</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>9048.833817999999</v>
+        <v>640362.403425</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>0</v>
+        <v>503515</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>-9048.833817999999</v>
+        <v>-136847.403425</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T521V107M016ATE050</t>
+          <t>T521D686M025ATE0707652</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>640362.403425</v>
+        <v>235515.668542</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>402758</v>
+        <v>33600</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>-237604.403425</v>
+        <v>-201915.668542</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>T521D686M025ATE0707652</t>
+          <t>T521D476M016ATE070</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>235515.668542</v>
+        <v>1055.302049</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>33600</v>
+        <v>0</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>-201915.668542</v>
+        <v>-1055.302049</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>T521D476M016ATE070</t>
+          <t>T598B107M006ATE045</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>1055.302049</v>
+        <v>549918.708952</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>0</v>
+        <v>456515</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>-1055.302049</v>
+        <v>-93403.70895200002</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>T598B107M006ATE045</t>
+          <t>T520D227M010ATE025</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>549918.708952</v>
+        <v>134086.464404</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>101295</v>
+        <v>33543</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>-448623.708952</v>
+        <v>-100543.464404</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>T598D337M006AT4143</t>
+          <t>T520D227M010ATE0257111</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>44748.0079</v>
+        <v>17900.546616</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>40584</v>
+        <v>0</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>-4164.007899999997</v>
+        <v>-17900.546616</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>T520D227M010ATE025</t>
+          <t>T520D477M004ATE012</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>134086.464404</v>
+        <v>108143.08831</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>33543</v>
+        <v>0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>-100543.464404</v>
+        <v>-108143.08831</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>T520D227M010ATE0257111</t>
+          <t>T521D157M025ATE050</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>17900.546616</v>
+        <v>3747</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>-17900.546616</v>
+        <v>-3747</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>T520D477M004ATE012</t>
+          <t>T520D687M004ATE012</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>108143.08831</v>
+        <v>37465.71564</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>-108143.08831</v>
+        <v>-37465.71564</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>T521D157M025ATE050</t>
+          <t>T521D227M016ATE050</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>3747</v>
+        <v>21571.717732</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>-3747</v>
+        <v>-21571.717732</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>T520D687M004ATE012</t>
+          <t>T521D107M020ATE055</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>37465.71564</v>
+        <v>225111.22586</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>-37465.71564</v>
+        <v>-225111.22586</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>T521D227M016ATE050</t>
+          <t>T521D476M020ATE055</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>21571.717732</v>
+        <v>55607.182309</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>-21571.717732</v>
+        <v>-55607.182309</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>T521D107M020ATE055</t>
+          <t>T525D476M016ATE065</t>
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>225111.22586</v>
+        <v>44850.337064</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>-225111.22586</v>
+        <v>-44850.337064</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>T521D476M020ATE055</t>
+          <t>T521D157M025ATE040</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>55607.182309</v>
+        <v>1249</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>-55607.182309</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>T525D476M016ATE065</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>44850.337064</v>
-      </c>
-      <c r="C22" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>-44850.337064</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>T521D157M025ATE040</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>1249</v>
-      </c>
-      <c r="C23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="1" t="n">
         <v>-1249</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add category column and switch to the latest uploaded planning data
- excel_shortage_analysis.py: read a new --category-mapping Anode
  workbook (Anode_Tantalum_Mapping sheet, COMP_ITEM -> Category) and
  prepend a category column before partNumber in both output sheets.
- Swap in the newly uploaded inputs (Anode 3-4-8.19.xlsx, Loading
  Aug.19th-New.xlsx, PlanningResult.xlsx, planningWarningMessage.xlsx)
  and regenerate shortage_report.xlsx from them.
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -417,32 +417,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>partNumber</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>202628</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>202634</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>matchedQty</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>gap</t>
         </is>
@@ -451,545 +457,892 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T520D157M010ATE040</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>3266.536296</v>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>T598D687M2R5ATE006</t>
+        </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>0</v>
+        <v>1060299.169066</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>-3266.536296</v>
+        <v>926843</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>-133456.169066</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T520D227M006ATE009E006</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>547.5072</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>T520V337M2R5ATE025</t>
+        </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0</v>
+        <v>15447.605017</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>-547.5072</v>
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>-15447.605017</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T520D477M004ATE0254539</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>2352.750189</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>T520D337M006ATE018</t>
+        </is>
       </c>
       <c r="C4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>-2352.750189</v>
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T598X477M010ATE025</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>1373.4396</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>T520D157M006ATE009E007</t>
+        </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0</v>
+        <v>1637.736953</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>-1373.4396</v>
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>-1637.736953</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T521D107M025ATE0407280</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>0</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>1269136</v>
+        <v>181558.102884</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>1269136</v>
+        <v>131718</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>-49840.10288399999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T520V337M2R5ATE007</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>0</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>T520D227M010ATE018</t>
+        </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>128798</v>
+        <v>0</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>128798</v>
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T520D337M006ATE009</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>636322.097301</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>T520B227M006ATE035</t>
+        </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>857390</v>
+        <v>0</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>221067.902699</v>
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T520D477M004ATE010</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>181559.085912</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T520B107M006ATE018</t>
+        </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>164687</v>
+        <v>5015.32295</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>-16872.08591199998</v>
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>-5015.32295</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>T520D337M006ATE040</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>9048.833817999999</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>T520V107M006ATE009E007</t>
+        </is>
       </c>
       <c r="C10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>-9048.833817999999</v>
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>T520W477M006ATE035</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>0</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>T520D337M006ATE009</t>
+        </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>23369</v>
+        <v>0</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>23369</v>
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>T521V107M016ATE050</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>640362.403425</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T521D227M016ATE035</t>
+        </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>503515</v>
+        <v>0</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>-136847.403425</v>
+        <v>0</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>T521D686M025ATE0707652</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>235515.668542</v>
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>T598D477M2R5ATE0067280</t>
+        </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>33600</v>
+        <v>0</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>-201915.668542</v>
+        <v>0</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>T521D476M016ATE070</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>1055.302049</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>T520V477M006ATE055</t>
+        </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>0</v>
+        <v>1361.377465</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>-1055.302049</v>
+        <v>0</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>-1361.377465</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>T591D226M025ATE060</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>0</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>T520B227M2R5ATE015</t>
+        </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>16518</v>
+        <v>0</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>16518</v>
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>T598B107M006ATE045</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>549918.708952</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>T520D477M004ATE012</t>
+        </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>456515</v>
+        <v>0</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>-93403.70895200002</v>
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>T598B686M006ATE070</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>0</v>
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>T521D107M025ATE0407280</t>
+        </is>
       </c>
       <c r="C17" s="1" t="n">
-        <v>0</v>
+        <v>3948929.81405</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>0</v>
+        <v>1499228</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>-2449701.81405</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>T598D337M006AT4143</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>44748.0079</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>T520V107M010ATE018</t>
+        </is>
       </c>
       <c r="C18" s="1" t="n">
-        <v>100225</v>
+        <v>115756.818077</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>55476.9921</v>
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>-115756.818077</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>T520D227M010ATE025</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>134086.464404</v>
+          <t>T59V</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>T521V107M020ATE055</t>
+        </is>
       </c>
       <c r="C19" s="1" t="n">
-        <v>33543</v>
+        <v>0</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>-100543.464404</v>
+        <v>797722</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>797722</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>T520D227M010ATE0257111</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>17900.546616</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>T520V477M006ATE035</t>
+        </is>
       </c>
       <c r="C20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>-17900.546616</v>
+        <v>0</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>T520D477M004ATE012</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>108143.08831</v>
+          <t>T528B</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>T528B277M002APE006</t>
+        </is>
       </c>
       <c r="C21" s="1" t="n">
-        <v>0</v>
+        <v>185610.378537</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>-108143.08831</v>
+        <v>0</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>-185610.378537</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>T521D157M025ATE050</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>3747</v>
+          <t>T528Z 1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>T528Z477M2R5ATE009E008</t>
+        </is>
       </c>
       <c r="C22" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>-3747</v>
+        <v>67184</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>67184</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>T520D687M004ATE012</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>37465.71564</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>T521B106M035ATE200</t>
+        </is>
       </c>
       <c r="C23" s="1" t="n">
-        <v>0</v>
+        <v>8786.043369999999</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>-37465.71564</v>
+        <v>0</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>-8786.043369999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>T521D227M016ATE050</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="n">
-        <v>21571.717732</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>T530D477M2R5ATE005</t>
+        </is>
       </c>
       <c r="C24" s="1" t="n">
-        <v>0</v>
+        <v>5421.686748</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>-21571.717732</v>
+        <v>0</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>-5421.686748</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>T521D107M020ATE055</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="n">
-        <v>225111.22586</v>
+          <t>T59V</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>T521V107M016ATE040</t>
+        </is>
       </c>
       <c r="C25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>-225111.22586</v>
+        <v>0</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>T521D476M020ATE055</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="n">
-        <v>55607.182309</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>T530X477M006ATE004</t>
+        </is>
       </c>
       <c r="C26" s="1" t="n">
-        <v>0</v>
+        <v>30835.536948</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>-55607.182309</v>
+        <v>0</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>-30835.536948</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>T525D476M016ATE065</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="n">
-        <v>44850.337064</v>
+          <t>2.0V</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>T521V476M016ATE040</t>
+        </is>
       </c>
       <c r="C27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>-44850.337064</v>
+        <v>0</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>T521D157M025ATE040</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="n">
-        <v>1249</v>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>T598D477M2R5ATE006</t>
+        </is>
       </c>
       <c r="C28" s="1" t="n">
-        <v>0</v>
+        <v>1209358.95066</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>-1249</v>
+        <v>591038</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>-618320.9506600001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>T520B337M2R5ATE015</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="n">
-        <v>190.207421</v>
+          <t>T59V</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>T521V157M016ATE050</t>
+        </is>
       </c>
       <c r="C29" s="1" t="n">
-        <v>51217</v>
+        <v>0</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>51026.792579</v>
+        <v>0</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>T520V477M2R5ATE007</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>9817.246623000001</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>T521X226M063ATE075</t>
+        </is>
       </c>
       <c r="C30" s="1" t="n">
-        <v>33587</v>
+        <v>0</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>23769.753377</v>
+        <v>0</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>T521V107M020ATE055</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="n">
-        <v>48497.818672</v>
+          <t>2.0V</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>T521V476M016ATE070</t>
+        </is>
       </c>
       <c r="C31" s="1" t="n">
-        <v>1065023</v>
+        <v>31567.049544</v>
       </c>
       <c r="D31" s="1" t="n">
-        <v>1016525.181328</v>
+        <v>0</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>-31567.049544</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>T521W476M020ATE045</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="n">
-        <v>13187.258162</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>T521X477M016ATE020</t>
+        </is>
       </c>
       <c r="C32" s="1" t="n">
-        <v>23558</v>
+        <v>107154.090896</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>10370.741838</v>
+        <v>0</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>-107154.090896</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>T530X337M010ATE010</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="n">
-        <v>0</v>
+          <t>T528Z 1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T528Z337M2R5ATE009E008</t>
+        </is>
       </c>
       <c r="C33" s="1" t="n">
-        <v>268459</v>
+        <v>0</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>268459</v>
+        <v>0</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>T530X158M2R5ATE005</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="n">
-        <v>0</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>T520B227M006ATE045</t>
+        </is>
       </c>
       <c r="C34" s="1" t="n">
-        <v>499420</v>
+        <v>0</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>499420</v>
+        <v>102000</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>102000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>T520X337M010ATE010</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>268557</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>268557</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>T530X337M010ATE004</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>7492.265061</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>-7492.265061</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>T530X687M004ATE004</t>
         </is>
       </c>
-      <c r="B35" s="1" t="n">
-        <v>32826.842256</v>
-      </c>
-      <c r="C35" s="1" t="n">
-        <v>33526</v>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>699.1577440000037</v>
+      <c r="C37" s="1" t="n">
+        <v>15400.177233</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>-15400.177233</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>T598D477M2R5AT4186</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="n">
+        <v>36969.354132</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>-36969.354132</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>T530X337M010AHE006</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>5101.127334000001</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>-5101.127334000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>T520V107M010ATE0502478</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="n">
+        <v>5669.429191</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>-5669.429191</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>T520V107M010ATE025</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="n">
+        <v>10131.826318</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>45066</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>34934.173682</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>T520B107M006ATE025</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>297872.79306</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>304191</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>6318.206940000004</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>T521D107M025ATE040</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="n">
+        <v>139986.564337</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>115534</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>-24452.56433700002</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>T530X337M010ATE005</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>68379</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>66593</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>-1786</v>
       </c>
     </row>
   </sheetData>
@@ -1003,32 +1356,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>partNumber</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>202628</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>202634</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>matchedQty</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>gap</t>
         </is>
@@ -1037,321 +1396,455 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T520D157M010ATE040</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>3266.536296</v>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>T598D687M2R5ATE006</t>
+        </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>0</v>
+        <v>1060299.169066</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>-3266.536296</v>
+        <v>926843</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>-133456.169066</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T520D227M006ATE009E006</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>547.5072</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>T520V337M2R5ATE025</t>
+        </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0</v>
+        <v>15447.605017</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>-547.5072</v>
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>-15447.605017</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T520D477M004ATE0254539</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>2352.750189</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>T520D157M006ATE009E007</t>
+        </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0</v>
+        <v>1637.736953</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>-2352.750189</v>
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>-1637.736953</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T598X477M010ATE025</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>1373.4396</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0</v>
+        <v>181558.102884</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>-1373.4396</v>
+        <v>131718</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>-49840.10288399999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T520D477M004ATE010</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>181559.085912</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>T520B107M006ATE018</t>
+        </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>164687</v>
+        <v>5015.32295</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>-16872.08591199998</v>
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>-5015.32295</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T520D337M006ATE040</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>9048.833817999999</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>T520V477M006ATE055</t>
+        </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>0</v>
+        <v>1361.377465</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>-9048.833817999999</v>
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>-1361.377465</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>T521V107M016ATE050</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>640362.403425</v>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>T521D107M025ATE0407280</t>
+        </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>503515</v>
+        <v>3948929.81405</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>-136847.403425</v>
+        <v>1499228</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>-2449701.81405</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T521D686M025ATE0707652</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>235515.668542</v>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T520V107M010ATE018</t>
+        </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>33600</v>
+        <v>115756.818077</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>-201915.668542</v>
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>-115756.818077</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>T521D476M016ATE070</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>1055.302049</v>
+          <t>T528B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>T528B277M002APE006</t>
+        </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>0</v>
+        <v>185610.378537</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>-1055.302049</v>
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>-185610.378537</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>T598B107M006ATE045</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>549918.708952</v>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>T521B106M035ATE200</t>
+        </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>456515</v>
+        <v>8786.043369999999</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>-93403.70895200002</v>
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-8786.043369999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>T520D227M010ATE025</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>134086.464404</v>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T530D477M2R5ATE005</t>
+        </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>33543</v>
+        <v>5421.686748</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>-100543.464404</v>
+        <v>0</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>-5421.686748</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>T520D227M010ATE0257111</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>17900.546616</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>T530X477M006ATE004</t>
+        </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>0</v>
+        <v>30835.536948</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>-17900.546616</v>
+        <v>0</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>-30835.536948</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>T520D477M004ATE012</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>108143.08831</v>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>T598D477M2R5ATE006</t>
+        </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>0</v>
+        <v>1209358.95066</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>-108143.08831</v>
+        <v>591038</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>-618320.9506600001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>T521D157M025ATE050</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>3747</v>
+          <t>2.0V</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>T521V476M016ATE070</t>
+        </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>0</v>
+        <v>31567.049544</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>-3747</v>
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>-31567.049544</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>T520D687M004ATE012</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>37465.71564</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>T521X477M016ATE020</t>
+        </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>0</v>
+        <v>107154.090896</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>-37465.71564</v>
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>-107154.090896</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>T521D227M016ATE050</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>21571.717732</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>T530X337M010ATE004</t>
+        </is>
       </c>
       <c r="C17" s="1" t="n">
-        <v>0</v>
+        <v>7492.265061</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>-21571.717732</v>
+        <v>0</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>-7492.265061</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>T521D107M020ATE055</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>225111.22586</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>T530X687M004ATE004</t>
+        </is>
       </c>
       <c r="C18" s="1" t="n">
-        <v>0</v>
+        <v>15400.177233</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>-225111.22586</v>
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>-15400.177233</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>T521D476M020ATE055</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>55607.182309</v>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>T598D477M2R5AT4186</t>
+        </is>
       </c>
       <c r="C19" s="1" t="n">
-        <v>0</v>
+        <v>36969.354132</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>-55607.182309</v>
+        <v>0</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>-36969.354132</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>T525D476M016ATE065</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>44850.337064</v>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>T530X337M010AHE006</t>
+        </is>
       </c>
       <c r="C20" s="1" t="n">
-        <v>0</v>
+        <v>5101.127334000001</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>-44850.337064</v>
+        <v>0</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>-5101.127334000001</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>T521D157M025ATE040</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>1249</v>
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>T520V107M010ATE0502478</t>
+        </is>
       </c>
       <c r="C21" s="1" t="n">
-        <v>0</v>
+        <v>5669.429191</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>-1249</v>
+        <v>0</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>-5669.429191</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>T521D107M025ATE040</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>139986.564337</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>115534</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>-24452.56433700002</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>T530X337M010ATE005</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>68379</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>66593</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>-1786</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fall back to PARENT_ITEM for category lookup when COMP_ITEM has no match
Some target partNumbers (lot-suffixed ones) only appear as PARENT_ITEM
in the Anode_Tantalum_Mapping sheet, not COMP_ITEM, leaving their
category blank. Look up COMP_ITEM first (unchanged for existing
matches), then fall back to PARENT_ITEM.
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -686,7 +686,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>T59D 2</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>T598D477M2R5ATE0067280</t>
@@ -766,7 +770,11 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="B17" t="inlineStr">
         <is>
           <t>T521D107M025ATE0407280</t>
@@ -1245,7 +1253,11 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1.9V</t>
+        </is>
+      </c>
       <c r="B40" t="inlineStr">
         <is>
           <t>T520V107M010ATE0502478</t>
@@ -1520,7 +1532,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>T521D107M025ATE0407280</t>
@@ -1789,7 +1805,11 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1.9V</t>
+        </is>
+      </c>
       <c r="B21" t="inlineStr">
         <is>
           <t>T520V107M010ATE0502478</t>

</xml_diff>

<commit_message>
Fix category source: use Loading's KEMET_GOP_ATO_ANALYSIS_DAILY sheet
The Anode workbook's Anode_Tantalum_Mapping sheet had inconsistent
categories for the same part (154 conflicting duplicate keys), which
produced wrong values (e.g. "T59D 1" instead of "T59D 2"). The Loading
workbook's KEMET_GOP_ATO_ANALYSIS_DAILY sheet maps PARENT_ITEM to
Anode Category with zero conflicts across all 36k rows and covers
every target partNumber, so use that instead. Drops the now-unused
--category-mapping argument and Anode input file.
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -457,7 +457,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -919,7 +919,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1003,7 +1003,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1148,11 +1148,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>T520X337M010ATE010</t>
@@ -1171,7 +1167,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1192,7 +1188,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1213,7 +1209,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1234,7 +1230,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1339,7 +1335,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1408,7 +1404,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1618,7 +1614,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1639,7 +1635,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1660,7 +1656,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1702,7 +1698,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1723,7 +1719,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1744,7 +1740,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1765,7 +1761,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1786,7 +1782,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1849,7 +1845,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">

</xml_diff>

<commit_message>
Add Actual TPT column after gap
Averages adjusted_tpt from the Loading workbook's "Overall TPT" sheet
(ItemName matched to partNumber) for each target partNumber.
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -49,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -425,6 +426,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,6 +455,11 @@
           <t>gap</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Actual TPT</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -474,6 +481,9 @@
       <c r="E2" s="1" t="n">
         <v>-133456.169066</v>
       </c>
+      <c r="F2" s="2" t="n">
+        <v>21.47815950920245</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -495,6 +505,9 @@
       <c r="E3" s="1" t="n">
         <v>-15447.605017</v>
       </c>
+      <c r="F3" s="2" t="n">
+        <v>17.506</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -516,6 +529,9 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F4" s="2" t="n">
+        <v>16.84041666666666</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,6 +553,9 @@
       <c r="E5" s="1" t="n">
         <v>-1637.736953</v>
       </c>
+      <c r="F5" s="2" t="n">
+        <v>19.90666666666667</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -558,6 +577,9 @@
       <c r="E6" s="1" t="n">
         <v>-49840.10288399999</v>
       </c>
+      <c r="F6" s="2" t="n">
+        <v>17.50933884297521</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -579,6 +601,9 @@
       <c r="E7" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F7" s="2" t="n">
+        <v>14.43026041666667</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -600,6 +625,9 @@
       <c r="E8" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F8" s="2" t="n">
+        <v>13.60854166666667</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -621,6 +649,9 @@
       <c r="E9" s="1" t="n">
         <v>-5015.32295</v>
       </c>
+      <c r="F9" s="2" t="n">
+        <v>19.20604166666667</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -642,6 +673,9 @@
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F10" s="2" t="n">
+        <v>22.4775</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -663,6 +697,9 @@
       <c r="E11" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F11" s="2" t="n">
+        <v>18.59724550898204</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -684,6 +721,9 @@
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F12" s="2" t="n">
+        <v>16.085</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -705,6 +745,9 @@
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F13" s="2" t="n">
+        <v>19.5720942408377</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -726,6 +769,9 @@
       <c r="E14" s="1" t="n">
         <v>-1361.377465</v>
       </c>
+      <c r="F14" s="2" t="n">
+        <v>18.434</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -747,6 +793,9 @@
       <c r="E15" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F15" s="2" t="n">
+        <v>16.91601851851852</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -768,6 +817,9 @@
       <c r="E16" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F16" s="2" t="n">
+        <v>16.01483870967742</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -789,6 +841,9 @@
       <c r="E17" s="1" t="n">
         <v>-2449701.81405</v>
       </c>
+      <c r="F17" s="2" t="n">
+        <v>11.93435144609988</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -810,6 +865,7 @@
       <c r="E18" s="1" t="n">
         <v>-115756.818077</v>
       </c>
+      <c r="F18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -831,6 +887,9 @@
       <c r="E19" s="1" t="n">
         <v>797722</v>
       </c>
+      <c r="F19" s="2" t="n">
+        <v>15.04557425742575</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -852,6 +911,9 @@
       <c r="E20" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F20" s="2" t="n">
+        <v>19.46818181818182</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -873,6 +935,9 @@
       <c r="E21" s="1" t="n">
         <v>-185610.378537</v>
       </c>
+      <c r="F21" s="2" t="n">
+        <v>36.352</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -894,6 +959,9 @@
       <c r="E22" s="1" t="n">
         <v>67184</v>
       </c>
+      <c r="F22" s="2" t="n">
+        <v>33.7525</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -915,6 +983,7 @@
       <c r="E23" s="1" t="n">
         <v>-8786.043369999999</v>
       </c>
+      <c r="F23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -936,6 +1005,9 @@
       <c r="E24" s="1" t="n">
         <v>-5421.686748</v>
       </c>
+      <c r="F24" s="2" t="n">
+        <v>19.66</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -957,6 +1029,9 @@
       <c r="E25" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F25" s="2" t="n">
+        <v>15.12</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -978,6 +1053,9 @@
       <c r="E26" s="1" t="n">
         <v>-30835.536948</v>
       </c>
+      <c r="F26" s="2" t="n">
+        <v>18.8862</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -999,6 +1077,9 @@
       <c r="E27" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F27" s="2" t="n">
+        <v>12.52</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1020,6 +1101,9 @@
       <c r="E28" s="1" t="n">
         <v>-618320.9506600001</v>
       </c>
+      <c r="F28" s="2" t="n">
+        <v>19.67699029126213</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1041,6 +1125,9 @@
       <c r="E29" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F29" s="2" t="n">
+        <v>17.25547619047619</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1062,6 +1149,9 @@
       <c r="E30" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F30" s="2" t="n">
+        <v>20.32785714285714</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1083,6 +1173,9 @@
       <c r="E31" s="1" t="n">
         <v>-31567.049544</v>
       </c>
+      <c r="F31" s="2" t="n">
+        <v>14.37666666666667</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1104,6 +1197,9 @@
       <c r="E32" s="1" t="n">
         <v>-107154.090896</v>
       </c>
+      <c r="F32" s="2" t="n">
+        <v>17.16212765957447</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1125,6 +1221,9 @@
       <c r="E33" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F33" s="2" t="n">
+        <v>33.815</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1145,6 +1244,9 @@
       </c>
       <c r="E34" s="1" t="n">
         <v>102000</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>13.93418198529412</v>
       </c>
     </row>
     <row r="35">
@@ -1163,6 +1265,7 @@
       <c r="E35" s="1" t="n">
         <v>268557</v>
       </c>
+      <c r="F35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1184,6 +1287,9 @@
       <c r="E36" s="1" t="n">
         <v>-7492.265061</v>
       </c>
+      <c r="F36" s="2" t="n">
+        <v>20.47947368421053</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1205,6 +1311,9 @@
       <c r="E37" s="1" t="n">
         <v>-15400.177233</v>
       </c>
+      <c r="F37" s="2" t="n">
+        <v>22.53768115942029</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1226,6 +1335,9 @@
       <c r="E38" s="1" t="n">
         <v>-36969.354132</v>
       </c>
+      <c r="F38" s="2" t="n">
+        <v>20.37757575757576</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1247,6 +1359,9 @@
       <c r="E39" s="1" t="n">
         <v>-5101.127334000001</v>
       </c>
+      <c r="F39" s="2" t="n">
+        <v>18.875</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1268,6 +1383,7 @@
       <c r="E40" s="1" t="n">
         <v>-5669.429191</v>
       </c>
+      <c r="F40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1289,6 +1405,9 @@
       <c r="E41" s="1" t="n">
         <v>34934.173682</v>
       </c>
+      <c r="F41" s="2" t="n">
+        <v>18.425</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1310,6 +1429,9 @@
       <c r="E42" s="1" t="n">
         <v>6318.206940000004</v>
       </c>
+      <c r="F42" s="2" t="n">
+        <v>12.53888888888889</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1331,6 +1453,9 @@
       <c r="E43" s="1" t="n">
         <v>-24452.56433700002</v>
       </c>
+      <c r="F43" s="2" t="n">
+        <v>12.48259717314488</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1351,6 +1476,9 @@
       </c>
       <c r="E44" s="1" t="n">
         <v>-1786</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>19.49571428571429</v>
       </c>
     </row>
   </sheetData>
@@ -1364,7 +1492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1372,6 +1500,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1400,6 +1529,11 @@
           <t>gap</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Actual TPT</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1421,6 +1555,9 @@
       <c r="E2" s="1" t="n">
         <v>-133456.169066</v>
       </c>
+      <c r="F2" s="2" t="n">
+        <v>21.47815950920245</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1442,6 +1579,9 @@
       <c r="E3" s="1" t="n">
         <v>-15447.605017</v>
       </c>
+      <c r="F3" s="2" t="n">
+        <v>17.506</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1463,6 +1603,9 @@
       <c r="E4" s="1" t="n">
         <v>-1637.736953</v>
       </c>
+      <c r="F4" s="2" t="n">
+        <v>19.90666666666667</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1484,6 +1627,9 @@
       <c r="E5" s="1" t="n">
         <v>-49840.10288399999</v>
       </c>
+      <c r="F5" s="2" t="n">
+        <v>17.50933884297521</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1505,6 +1651,9 @@
       <c r="E6" s="1" t="n">
         <v>-5015.32295</v>
       </c>
+      <c r="F6" s="2" t="n">
+        <v>19.20604166666667</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1526,6 +1675,9 @@
       <c r="E7" s="1" t="n">
         <v>-1361.377465</v>
       </c>
+      <c r="F7" s="2" t="n">
+        <v>18.434</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1547,6 +1699,9 @@
       <c r="E8" s="1" t="n">
         <v>-2449701.81405</v>
       </c>
+      <c r="F8" s="2" t="n">
+        <v>11.93435144609988</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1568,6 +1723,7 @@
       <c r="E9" s="1" t="n">
         <v>-115756.818077</v>
       </c>
+      <c r="F9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1589,6 +1745,9 @@
       <c r="E10" s="1" t="n">
         <v>-185610.378537</v>
       </c>
+      <c r="F10" s="2" t="n">
+        <v>36.352</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1610,6 +1769,7 @@
       <c r="E11" s="1" t="n">
         <v>-8786.043369999999</v>
       </c>
+      <c r="F11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1631,6 +1791,9 @@
       <c r="E12" s="1" t="n">
         <v>-5421.686748</v>
       </c>
+      <c r="F12" s="2" t="n">
+        <v>19.66</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1652,6 +1815,9 @@
       <c r="E13" s="1" t="n">
         <v>-30835.536948</v>
       </c>
+      <c r="F13" s="2" t="n">
+        <v>18.8862</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1673,6 +1839,9 @@
       <c r="E14" s="1" t="n">
         <v>-618320.9506600001</v>
       </c>
+      <c r="F14" s="2" t="n">
+        <v>19.67699029126213</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1694,6 +1863,9 @@
       <c r="E15" s="1" t="n">
         <v>-31567.049544</v>
       </c>
+      <c r="F15" s="2" t="n">
+        <v>14.37666666666667</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1715,6 +1887,9 @@
       <c r="E16" s="1" t="n">
         <v>-107154.090896</v>
       </c>
+      <c r="F16" s="2" t="n">
+        <v>17.16212765957447</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1736,6 +1911,9 @@
       <c r="E17" s="1" t="n">
         <v>-7492.265061</v>
       </c>
+      <c r="F17" s="2" t="n">
+        <v>20.47947368421053</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1757,6 +1935,9 @@
       <c r="E18" s="1" t="n">
         <v>-15400.177233</v>
       </c>
+      <c r="F18" s="2" t="n">
+        <v>22.53768115942029</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1778,6 +1959,9 @@
       <c r="E19" s="1" t="n">
         <v>-36969.354132</v>
       </c>
+      <c r="F19" s="2" t="n">
+        <v>20.37757575757576</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1799,6 +1983,9 @@
       <c r="E20" s="1" t="n">
         <v>-5101.127334000001</v>
       </c>
+      <c r="F20" s="2" t="n">
+        <v>18.875</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1820,6 +2007,7 @@
       <c r="E21" s="1" t="n">
         <v>-5669.429191</v>
       </c>
+      <c r="F21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1841,6 +2029,9 @@
       <c r="E22" s="1" t="n">
         <v>-24452.56433700002</v>
       </c>
+      <c r="F22" s="2" t="n">
+        <v>12.48259717314488</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1861,6 +2052,9 @@
       </c>
       <c r="E23" s="1" t="n">
         <v>-1786</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>19.49571428571429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>